<commit_message>
Add Status column to dispatch dashboard, include Suchitra in route map
</commit_message>
<xml_diff>
--- a/ghmc-routing/output/ghmc_route_map.xlsx
+++ b/ghmc-routing/output/ghmc_route_map.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GHMC Route Map" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'GHMC Route Map'!$A$1:$H$422</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'GHMC Route Map'!$A$1:$H$424</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'GHMC Route Map'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H422"/>
+  <dimension ref="A1:H424"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.8" customWidth="1" min="1" max="1"/>
@@ -16249,229 +16249,229 @@
     <row r="416">
       <c r="A416" s="2" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B416" s="2" t="inlineStr">
         <is>
-          <t>South-West (SW) Route</t>
+          <t>North-West (NW) Route</t>
         </is>
       </c>
       <c r="C416" s="2" t="inlineStr">
         <is>
-          <t>Serilingampally Zone - South-West Belt</t>
+          <t>Kukatpally/Quthbullapur Zone - North-West Wings</t>
         </is>
       </c>
       <c r="D416" s="2" t="inlineStr">
         <is>
-          <t>Serilingampally</t>
+          <t>Jeedimetla</t>
         </is>
       </c>
       <c r="E416" s="2" t="inlineStr">
         <is>
-          <t>- (locality): Gcachibowli</t>
+          <t>- (locality): Suchitra</t>
         </is>
       </c>
       <c r="F416" s="2" t="inlineStr">
         <is>
-          <t>Alt. spelling of Gachibowli; ORR tech belt; deliver 11 AM-4 PM.</t>
+          <t>Quthbullapur residential circle on the ring road (north of Jeedimetla); gated layouts; combine Jeedimetla return loop.</t>
         </is>
       </c>
       <c r="G416" s="2" t="n">
-        <v>17.466717</v>
+        <v>17.519687</v>
       </c>
       <c r="H416" s="2" t="n">
-        <v>78.34042100000001</v>
+        <v>78.446888</v>
       </c>
     </row>
     <row r="417">
       <c r="A417" s="3" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="B417" s="3" t="inlineStr">
         <is>
-          <t>North-West (NW) Route</t>
+          <t>South-West (SW) Route</t>
         </is>
       </c>
       <c r="C417" s="3" t="inlineStr">
         <is>
-          <t>Kukatpally Zone - North-West Wing</t>
+          <t>Serilingampally Zone - South-West Belt</t>
         </is>
       </c>
       <c r="D417" s="3" t="inlineStr">
         <is>
-          <t>Kukatpally</t>
+          <t>Serilingampally</t>
         </is>
       </c>
       <c r="E417" s="3" t="inlineStr">
         <is>
-          <t>- (locality): Kkatpally</t>
+          <t>- (locality): Gcachibowli</t>
         </is>
       </c>
       <c r="F417" s="3" t="inlineStr">
         <is>
-          <t>Alt. spelling of Kukatpally; KPHB high-density; 6-10 AM window.</t>
+          <t>Alt. spelling of Gachibowli; ORR tech belt; deliver 11 AM-4 PM.</t>
         </is>
       </c>
       <c r="G417" s="3" t="n">
-        <v>17.493084</v>
+        <v>17.466717</v>
       </c>
       <c r="H417" s="3" t="n">
-        <v>78.405441</v>
+        <v>78.34042100000001</v>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B418" s="2" t="inlineStr">
         <is>
-          <t>South-East (SE) Route</t>
+          <t>North-West (NW) Route</t>
         </is>
       </c>
       <c r="C418" s="2" t="inlineStr">
         <is>
-          <t>Charminar Zone - South-East Belt</t>
+          <t>Kukatpally Zone - North-West Wing</t>
         </is>
       </c>
       <c r="D418" s="2" t="inlineStr">
         <is>
-          <t>Malakpet</t>
+          <t>Kukatpally</t>
         </is>
       </c>
       <c r="E418" s="2" t="inlineStr">
         <is>
-          <t>- (locality): Malkpet</t>
+          <t>- (locality): Kkatpally</t>
         </is>
       </c>
       <c r="F418" s="2" t="inlineStr">
         <is>
-          <t>Alt. spelling of Malakpet; commercial mid-belt; post-11 AM.</t>
+          <t>Alt. spelling of Kukatpally; KPHB high-density; 6-10 AM window.</t>
         </is>
       </c>
       <c r="G418" s="2" t="n">
-        <v>17.373671</v>
+        <v>17.493084</v>
       </c>
       <c r="H418" s="2" t="n">
-        <v>78.49964799999999</v>
+        <v>78.405441</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" s="3" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="B419" s="3" t="inlineStr">
         <is>
-          <t>South-West (SW) Route</t>
+          <t>South-East (SE) Route</t>
         </is>
       </c>
       <c r="C419" s="3" t="inlineStr">
         <is>
-          <t>Khairatabad Zone - Central-South Belt</t>
+          <t>Charminar Zone - South-East Belt</t>
         </is>
       </c>
       <c r="D419" s="3" t="inlineStr">
         <is>
-          <t>Mehdipatnam</t>
+          <t>Malakpet</t>
         </is>
       </c>
       <c r="E419" s="3" t="inlineStr">
         <is>
-          <t>- (locality): Mehndipatnam</t>
+          <t>- (locality): Malkpet</t>
         </is>
       </c>
       <c r="F419" s="3" t="inlineStr">
         <is>
-          <t>Alt. spelling of Mehdipatnam; market + residential; after 11 AM.</t>
+          <t>Alt. spelling of Malakpet; commercial mid-belt; post-11 AM.</t>
         </is>
       </c>
       <c r="G419" s="3" t="n">
-        <v>17.394263</v>
+        <v>17.373671</v>
       </c>
       <c r="H419" s="3" t="n">
-        <v>78.434251</v>
+        <v>78.49964799999999</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="B420" s="2" t="inlineStr">
         <is>
-          <t>North-West (NW) Route</t>
+          <t>South-West (SW) Route</t>
         </is>
       </c>
       <c r="C420" s="2" t="inlineStr">
         <is>
-          <t>Kukatpally Zone - North-West Wing</t>
+          <t>Khairatabad Zone - Central-South Belt</t>
         </is>
       </c>
       <c r="D420" s="2" t="inlineStr">
         <is>
-          <t>Miyapur</t>
+          <t>Mehdipatnam</t>
         </is>
       </c>
       <c r="E420" s="2" t="inlineStr">
         <is>
-          <t>- (locality): Myapur</t>
+          <t>- (locality): Mehndipatnam</t>
         </is>
       </c>
       <c r="F420" s="2" t="inlineStr">
         <is>
-          <t>Alt. spelling of Miyapur; NH65 corridor; mid-day.</t>
+          <t>Alt. spelling of Mehdipatnam; market + residential; after 11 AM.</t>
         </is>
       </c>
       <c r="G420" s="2" t="n">
-        <v>17.498161</v>
+        <v>17.394263</v>
       </c>
       <c r="H420" s="2" t="n">
-        <v>78.356763</v>
+        <v>78.434251</v>
       </c>
     </row>
     <row r="421">
       <c r="A421" s="3" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B421" s="3" t="inlineStr">
         <is>
-          <t>South-West (SW) Route</t>
+          <t>North-West (NW) Route</t>
         </is>
       </c>
       <c r="C421" s="3" t="inlineStr">
         <is>
-          <t>Serilingampally Zone - South-West Belt</t>
+          <t>Kukatpally Zone - North-West Wing</t>
         </is>
       </c>
       <c r="D421" s="3" t="inlineStr">
         <is>
-          <t>Madhapur</t>
+          <t>Miyapur</t>
         </is>
       </c>
       <c r="E421" s="3" t="inlineStr">
         <is>
-          <t>- (locality): Hitech City</t>
+          <t>- (locality): Myapur</t>
         </is>
       </c>
       <c r="F421" s="3" t="inlineStr">
         <is>
-          <t>Alt. spelling of HITEC City (ward 231); same routing as Madhapur.</t>
+          <t>Alt. spelling of Miyapur; NH65 corridor; mid-day.</t>
         </is>
       </c>
       <c r="G421" s="3" t="n">
-        <v>17.440892</v>
+        <v>17.498161</v>
       </c>
       <c r="H421" s="3" t="n">
-        <v>78.39163000000001</v>
+        <v>78.356763</v>
       </c>
     </row>
     <row r="422">
@@ -16487,33 +16487,109 @@
       </c>
       <c r="C422" s="2" t="inlineStr">
         <is>
+          <t>Serilingampally Zone - South-West Belt</t>
+        </is>
+      </c>
+      <c r="D422" s="2" t="inlineStr">
+        <is>
+          <t>Madhapur</t>
+        </is>
+      </c>
+      <c r="E422" s="2" t="inlineStr">
+        <is>
+          <t>- (locality): Hitech City</t>
+        </is>
+      </c>
+      <c r="F422" s="2" t="inlineStr">
+        <is>
+          <t>Alt. spelling of HITEC City (ward 231); same routing as Madhapur.</t>
+        </is>
+      </c>
+      <c r="G422" s="2" t="n">
+        <v>17.440892</v>
+      </c>
+      <c r="H422" s="2" t="n">
+        <v>78.39163000000001</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="3" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B423" s="3" t="inlineStr">
+        <is>
+          <t>South-West (SW) Route</t>
+        </is>
+      </c>
+      <c r="C423" s="3" t="inlineStr">
+        <is>
           <t>Khairatabad Zone - Central-South Belt</t>
         </is>
       </c>
-      <c r="D422" s="2" t="inlineStr">
+      <c r="D423" s="3" t="inlineStr">
         <is>
           <t>Khairatabad</t>
         </is>
       </c>
-      <c r="E422" s="2" t="inlineStr">
+      <c r="E423" s="3" t="inlineStr">
         <is>
           <t>- (locality): Himayatnagar</t>
         </is>
       </c>
-      <c r="F422" s="2" t="inlineStr">
+      <c r="F423" s="3" t="inlineStr">
         <is>
           <t>Alt. spelling of Himayathnagar (ward 220); central corporate; 10 AM-5 PM.</t>
         </is>
       </c>
-      <c r="G422" s="2" t="n">
+      <c r="G423" s="3" t="n">
         <v>17.412974</v>
       </c>
-      <c r="H422" s="2" t="n">
+      <c r="H423" s="3" t="n">
         <v>78.46105799999999</v>
       </c>
     </row>
+    <row r="424">
+      <c r="A424" s="2" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B424" s="2" t="inlineStr">
+        <is>
+          <t>North-West (NW) Route</t>
+        </is>
+      </c>
+      <c r="C424" s="2" t="inlineStr">
+        <is>
+          <t>Kukatpally/Quthbullapur Zone - North-West Wings</t>
+        </is>
+      </c>
+      <c r="D424" s="2" t="inlineStr">
+        <is>
+          <t>Jeedimetla</t>
+        </is>
+      </c>
+      <c r="E424" s="2" t="inlineStr">
+        <is>
+          <t>- (locality): Suchitra Circle</t>
+        </is>
+      </c>
+      <c r="F424" s="2" t="inlineStr">
+        <is>
+          <t>Alt. spelling of Suchitra; Quthbullapur residential circle; combine Jeedimetla return loop.</t>
+        </is>
+      </c>
+      <c r="G424" s="2" t="n">
+        <v>17.519687</v>
+      </c>
+      <c r="H424" s="2" t="n">
+        <v>78.446888</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H422"/>
+  <autoFilter ref="A1:H424"/>
   <printOptions gridLines="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>